<commit_message>
Update tfr postplanner 2026-04-06 xlsx and pycache
https://claude.ai/code/session_01KNv36HtfZFXQRG72Mv5RF6
</commit_message>
<xml_diff>
--- a/Tennis/postplanner-imports/tfr-postplanner-2026-04-06.xlsx
+++ b/Tennis/postplanner-imports/tfr-postplanner-2026-04-06.xlsx
@@ -478,7 +478,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>04/06/2026  13:21</t>
+          <t>04/06/2026  08:00</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -490,7 +490,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>04/06/2026  14:25</t>
+          <t>04/06/2026  10:30</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -502,7 +502,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>04/06/2026  15:29</t>
+          <t>04/06/2026  12:30</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -514,7 +514,7 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>04/06/2026  16:33</t>
+          <t>04/06/2026  15:00</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -526,7 +526,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>04/06/2026  17:37</t>
+          <t>04/06/2026  15:05</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -538,7 +538,7 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>04/06/2026  18:41</t>
+          <t>04/06/2026  18:00</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -550,7 +550,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>04/06/2026  19:45</t>
+          <t>04/06/2026  18:05</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -562,7 +562,7 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>04/06/2026  20:49</t>
+          <t>04/06/2026  21:00</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">

</xml_diff>